<commit_message>
added Get Attribute and Tests for types I32,DBL,BOOL
</commit_message>
<xml_diff>
--- a/Source/Tests/Test Config From EXCEL/test_configurations.xlsx
+++ b/Source/Tests/Test Config From EXCEL/test_configurations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\HAL\Source\Tests\Test Config From EXCEL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71896C42-B876-4DED-8AFF-FDFD2B4F7BB3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B43F597-7F37-4C1B-A4D8-92FF5D44CA05}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7980" xr2:uid="{694A1011-F733-4B3D-865A-EAFA5EFA9CF7}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="7980" activeTab="2" xr2:uid="{694A1011-F733-4B3D-865A-EAFA5EFA9CF7}"/>
   </bookViews>
   <sheets>
     <sheet name="Instruments" sheetId="3" r:id="rId1"/>
@@ -82,9 +82,6 @@
     <t>Attributes.DbcFilepath</t>
   </si>
   <si>
-    <t>D:\\git\\HAL\\HAL-Devices\\Tests\\resources\\Triple-Sensor-NEO480.dbc</t>
-  </si>
-  <si>
     <t>Attributes.Termination</t>
   </si>
   <si>
@@ -92,6 +89,9 @@
   </si>
   <si>
     <t>Attributes.GrpcServerAddress</t>
+  </si>
+  <si>
+    <t>D:\git\HAL\HAL-Devices\Tests\resources\Triple-Sensor-NEO480.dbc</t>
   </si>
 </sst>
 </file>
@@ -180,7 +180,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -196,7 +196,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -493,7 +493,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBC1553D-31A9-47F1-9003-2533A43CD3A4}">
   <dimension ref="A1:A21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
   </cols>
@@ -575,7 +575,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6A9D403-72C5-472F-AC2B-4CAB762784A6}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.140625" customWidth="1"/>
     <col min="2" max="2" width="72.42578125" customWidth="1"/>
@@ -626,7 +626,7 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -638,7 +638,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A7DE5E1-2065-4857-A2CD-738C548B16E2}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.28515625" customWidth="1"/>
     <col min="2" max="2" width="72" customWidth="1"/>
@@ -681,7 +681,7 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>10</v>
+        <v>10.1</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -689,12 +689,12 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -702,10 +702,10 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>